<commit_message>
chore: full dashboard + campaign analysis refresh [2026-05-22]
Sent 2.58M · Contacted 941K · Interested 1675 · Demos 405 · Shows 226
Pending 31 · Closed 25 (ARR \$245,460).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cold_email_workflows/cold_email_insights/data/campaign_analysis.xlsx
+++ b/cold_email_workflows/cold_email_insights/data/campaign_analysis.xlsx
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Source: metrics.json generated 2026-05-21T22:06:09.167162Z</t>
+          <t>Source: metrics.json generated 2026-05-21T22:19:37.317935Z</t>
         </is>
       </c>
     </row>
@@ -2616,10 +2616,10 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>8024</v>
+        <v>8026</v>
       </c>
       <c r="G2" t="n">
-        <v>8024</v>
+        <v>8026</v>
       </c>
       <c r="H2" t="n">
         <v>172</v>
@@ -2680,10 +2680,10 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>5936</v>
+        <v>5941</v>
       </c>
       <c r="G3" t="n">
-        <v>5936</v>
+        <v>5941</v>
       </c>
       <c r="H3" t="n">
         <v>125</v>
@@ -2744,16 +2744,16 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>2896</v>
+        <v>2920</v>
       </c>
       <c r="G4" t="n">
-        <v>2896</v>
+        <v>2921</v>
       </c>
       <c r="H4" t="n">
         <v>7</v>
       </c>
       <c r="I4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J4" t="n">
         <v>2</v>
@@ -2808,13 +2808,13 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>16806</v>
+        <v>16982</v>
       </c>
       <c r="G5" t="n">
         <v>9715</v>
       </c>
       <c r="H5" t="n">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="I5" t="n">
         <v>132</v>
@@ -2872,13 +2872,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>11685</v>
+        <v>11802</v>
       </c>
       <c r="G6" t="n">
-        <v>6985</v>
+        <v>6986</v>
       </c>
       <c r="H6" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I6" t="n">
         <v>280</v>
@@ -2936,16 +2936,16 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>8474</v>
+        <v>8534</v>
       </c>
       <c r="G7" t="n">
-        <v>6351</v>
+        <v>6364</v>
       </c>
       <c r="H7" t="n">
         <v>39</v>
       </c>
       <c r="I7" t="n">
-        <v>1226</v>
+        <v>1234</v>
       </c>
       <c r="J7" t="n">
         <v>6</v>
@@ -3000,16 +3000,16 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>12879</v>
+        <v>12914</v>
       </c>
       <c r="G8" t="n">
-        <v>11819</v>
+        <v>11831</v>
       </c>
       <c r="H8" t="n">
         <v>30</v>
       </c>
       <c r="I8" t="n">
-        <v>1486</v>
+        <v>1492</v>
       </c>
       <c r="J8" t="n">
         <v>1</v>
@@ -3064,7 +3064,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>12585</v>
+        <v>12720</v>
       </c>
       <c r="G9" t="n">
         <v>7300</v>
@@ -3073,7 +3073,7 @@
         <v>112</v>
       </c>
       <c r="I9" t="n">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="J9" t="n">
         <v>3</v>
@@ -3128,10 +3128,10 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>17908</v>
+        <v>18057</v>
       </c>
       <c r="G10" t="n">
-        <v>12321</v>
+        <v>12322</v>
       </c>
       <c r="H10" t="n">
         <v>254</v>
@@ -3192,7 +3192,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>11253</v>
+        <v>11275</v>
       </c>
       <c r="G11" t="n">
         <v>6902</v>
@@ -3256,7 +3256,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>4904</v>
+        <v>4926</v>
       </c>
       <c r="G12" t="n">
         <v>2649</v>
@@ -3320,7 +3320,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="G13" t="n">
         <v>590</v>
@@ -3384,10 +3384,10 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1876</v>
+        <v>1891</v>
       </c>
       <c r="G14" t="n">
-        <v>1457</v>
+        <v>1461</v>
       </c>
       <c r="H14" t="n">
         <v>3</v>
@@ -3448,10 +3448,10 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>20922</v>
+        <v>20927</v>
       </c>
       <c r="G15" t="n">
-        <v>13337</v>
+        <v>13339</v>
       </c>
       <c r="H15" t="n">
         <v>89</v>
@@ -3512,7 +3512,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>23306</v>
+        <v>23311</v>
       </c>
       <c r="G16" t="n">
         <v>8191</v>
@@ -3576,7 +3576,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>10146</v>
+        <v>10166</v>
       </c>
       <c r="G17" t="n">
         <v>3687</v>
@@ -3768,7 +3768,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>23874</v>
+        <v>23901</v>
       </c>
       <c r="G20" t="n">
         <v>8366</v>
@@ -3832,7 +3832,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>11802</v>
+        <v>11810</v>
       </c>
       <c r="G21" t="n">
         <v>4505</v>
@@ -3896,7 +3896,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2035</v>
+        <v>2043</v>
       </c>
       <c r="G22" t="n">
         <v>1127</v>
@@ -3960,7 +3960,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>6147</v>
+        <v>6154</v>
       </c>
       <c r="G23" t="n">
         <v>4876</v>
@@ -4088,7 +4088,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>16287</v>
+        <v>16292</v>
       </c>
       <c r="G25" t="n">
         <v>5743</v>
@@ -4152,10 +4152,10 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2001</v>
+        <v>2011</v>
       </c>
       <c r="G26" t="n">
-        <v>1358</v>
+        <v>1361</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -4216,10 +4216,10 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>5244</v>
+        <v>5247</v>
       </c>
       <c r="G27" t="n">
-        <v>4728</v>
+        <v>4730</v>
       </c>
       <c r="H27" t="n">
         <v>14</v>
@@ -4280,7 +4280,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>13709</v>
+        <v>13710</v>
       </c>
       <c r="G28" t="n">
         <v>6177</v>
@@ -4472,7 +4472,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>20539</v>
+        <v>20540</v>
       </c>
       <c r="G31" t="n">
         <v>7260</v>
@@ -4536,7 +4536,7 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>44480</v>
+        <v>44483</v>
       </c>
       <c r="G32" t="n">
         <v>19301</v>
@@ -4600,7 +4600,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>7646</v>
+        <v>7651</v>
       </c>
       <c r="G33" t="n">
         <v>3168</v>
@@ -4984,7 +4984,7 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>3808</v>
+        <v>3810</v>
       </c>
       <c r="G39" t="n">
         <v>2687</v>
@@ -5112,7 +5112,7 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>12609</v>
+        <v>12618</v>
       </c>
       <c r="G41" t="n">
         <v>4369</v>
@@ -5176,7 +5176,7 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>46965</v>
+        <v>46978</v>
       </c>
       <c r="G42" t="n">
         <v>14868</v>
@@ -5240,7 +5240,7 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>408081</v>
+        <v>408313</v>
       </c>
       <c r="G43" t="n">
         <v>133975</v>
@@ -5304,7 +5304,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>205523</v>
+        <v>205525</v>
       </c>
       <c r="G44" t="n">
         <v>56079</v>
@@ -5368,7 +5368,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>176301</v>
+        <v>176303</v>
       </c>
       <c r="G45" t="n">
         <v>45638</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>57888</v>
+        <v>57922</v>
       </c>
       <c r="G46" t="n">
         <v>17546</v>

</xml_diff>